<commit_message>
mise à jour du portfolio et des docuemnts
</commit_message>
<xml_diff>
--- a/public/e5/annexe8-1_tableau_synthese.xlsx
+++ b/public/e5/annexe8-1_tableau_synthese.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\frani\OneDrive\Bureau\project\public\e5\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\frani\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12D55A7E-9A52-4EF3-9624-37736FAC25D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2378B660-F7BC-4B39-9EBB-DA810F1C700D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
   <si>
     <t>Gérer le patrimoine informatique</t>
   </si>
@@ -101,9 +101,6 @@
 (intitulé et liste des documents et productions associés)</t>
   </si>
   <si>
-    <t xml:space="preserve">N° candidat : </t>
-  </si>
-  <si>
     <t>Période (sous la forme du JJ/MM/AA au JJ/MM/AA)</t>
   </si>
   <si>
@@ -122,18 +119,6 @@
     <t>Linkedin www.linkedin.com/in/tinofranic</t>
   </si>
   <si>
-    <t>Mission 1 : Restructuration de l'Infrastructure de StadiumCompany</t>
-  </si>
-  <si>
-    <t>Mission 2 : Infrastructure, Configuration et Administration</t>
-  </si>
-  <si>
-    <t>Mission 3 : Mise en Place d'une Solution pour l'Administration</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Elaboration d'une veille technologique sur la 6G</t>
-  </si>
-  <si>
     <t>Assistance aux utilisateurs</t>
   </si>
   <si>
@@ -174,6 +159,34 @@
   </si>
   <si>
     <t>Gestion des commandes de téléphones et forfaits</t>
+  </si>
+  <si>
+    <t>N° candidat : 2544739731</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Elaboration de veille Technologique</t>
+  </si>
+  <si>
+    <t>Restructuration de l'infrastructure Stadium company (VLAN, VTP, 
+Routage inter-vlan, Routage Statique)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Infrastructure, Configuration et Administration des Services
+ Informatiques de Stadium (Active Directory) </t>
+  </si>
+  <si>
+    <t>Mise en Place d'une Solution pour l'Administration à Distance Sécurisée et la Sécurisation des Interconnexions (SSH, VPN)</t>
+  </si>
+  <si>
+    <t>Solution de redondance, tolérance de panne et équilibrage de charge 
+pour les équipements réseau (HSRP, spannning-tree)</t>
+  </si>
+  <si>
+    <t>Sécurisation de l'Interconnexion du Réseau de Stadium avec Internet 
+(PfSense)</t>
+  </si>
+  <si>
+    <t>010/02/2025</t>
   </si>
 </sst>
 </file>
@@ -290,7 +303,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="25">
+  <borders count="26">
     <border>
       <left/>
       <right/>
@@ -612,10 +625,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="2" tint="-0.749992370372631"/>
+      </left>
+      <right style="thin">
+        <color theme="2" tint="-0.749992370372631"/>
+      </right>
+      <top style="thin">
+        <color theme="2" tint="-0.749992370372631"/>
+      </top>
+      <bottom style="thin">
+        <color theme="2" tint="-0.749992370372631"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -655,7 +684,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -669,9 +697,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -685,9 +710,6 @@
     <xf numFmtId="14" fontId="4" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -697,9 +719,43 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -724,44 +780,20 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="25" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Euro" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="2" xr:uid="{77714221-6730-42E1-A7B4-CC892D6DA250}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1191,7 +1223,7 @@
       <c r="E1" s="29"/>
       <c r="F1" s="29"/>
       <c r="G1" s="29" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H1" s="29"/>
     </row>
@@ -1208,30 +1240,30 @@
       <c r="H2" s="29"/>
     </row>
     <row r="3" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="30" t="s">
-        <v>24</v>
-      </c>
-      <c r="B3" s="31"/>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="36" t="s">
-        <v>19</v>
-      </c>
-      <c r="G3" s="31"/>
-      <c r="H3" s="37"/>
+      <c r="A3" s="39" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="40"/>
+      <c r="C3" s="40"/>
+      <c r="D3" s="40"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="45" t="s">
+        <v>39</v>
+      </c>
+      <c r="G3" s="40"/>
+      <c r="H3" s="46"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="33" t="s">
-        <v>36</v>
-      </c>
-      <c r="B4" s="34"/>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="35"/>
+      <c r="A4" s="42" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" s="43"/>
+      <c r="C4" s="43"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="44"/>
       <c r="F4" s="10" t="s">
         <v>8</v>
       </c>
@@ -1243,23 +1275,23 @@
       </c>
     </row>
     <row r="5" spans="1:43" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="46" t="s">
-        <v>37</v>
-      </c>
-      <c r="B5" s="47"/>
-      <c r="C5" s="47"/>
-      <c r="D5" s="47"/>
-      <c r="E5" s="47"/>
-      <c r="F5" s="47"/>
-      <c r="G5" s="47"/>
-      <c r="H5" s="48"/>
+      <c r="A5" s="36" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" s="37"/>
+      <c r="C5" s="37"/>
+      <c r="D5" s="37"/>
+      <c r="E5" s="37"/>
+      <c r="F5" s="37"/>
+      <c r="G5" s="37"/>
+      <c r="H5" s="38"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="38" t="s">
+      <c r="A6" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="44" t="s">
-        <v>20</v>
+      <c r="B6" s="34" t="s">
+        <v>19</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>0</v>
@@ -1281,15 +1313,15 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="324.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="39"/>
-      <c r="B7" s="45"/>
+      <c r="A7" s="28"/>
+      <c r="B7" s="35"/>
       <c r="C7" s="8" t="s">
         <v>9</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="28" t="s">
+      <c r="E7" s="25" t="s">
         <v>11</v>
       </c>
       <c r="F7" s="8" t="s">
@@ -1338,16 +1370,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A8" s="40" t="s">
+      <c r="A8" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="41"/>
-      <c r="C8" s="41"/>
-      <c r="D8" s="41"/>
-      <c r="E8" s="41"/>
-      <c r="F8" s="41"/>
-      <c r="G8" s="41"/>
-      <c r="H8" s="42"/>
+      <c r="B8" s="31"/>
+      <c r="C8" s="31"/>
+      <c r="D8" s="31"/>
+      <c r="E8" s="31"/>
+      <c r="F8" s="31"/>
+      <c r="G8" s="31"/>
+      <c r="H8" s="32"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1385,18 +1417,18 @@
       <c r="AQ8"/>
     </row>
     <row r="9" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="B9" s="24">
+      <c r="A9" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="22">
         <v>45689</v>
       </c>
-      <c r="C9" s="15"/>
-      <c r="D9" s="16"/>
-      <c r="E9" s="16"/>
-      <c r="F9" s="16"/>
-      <c r="G9" s="16"/>
-      <c r="H9" s="17"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="16"/>
       <c r="I9"/>
       <c r="J9"/>
       <c r="K9"/>
@@ -1434,18 +1466,18 @@
       <c r="AQ9"/>
     </row>
     <row r="10" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="B10" s="24">
+      <c r="A10" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" s="22">
         <v>45717</v>
       </c>
-      <c r="C10" s="16"/>
-      <c r="D10" s="16"/>
-      <c r="E10" s="16"/>
-      <c r="F10" s="16"/>
-      <c r="G10" s="16"/>
-      <c r="H10" s="17"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="15"/>
+      <c r="H10" s="16"/>
       <c r="I10"/>
       <c r="J10"/>
       <c r="K10"/>
@@ -1483,18 +1515,18 @@
       <c r="AQ10"/>
     </row>
     <row r="11" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="21" t="s">
-        <v>26</v>
-      </c>
-      <c r="B11" s="24">
+      <c r="A11" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="B11" s="22">
         <v>45913</v>
       </c>
-      <c r="C11" s="17"/>
-      <c r="D11" s="16"/>
-      <c r="E11" s="16"/>
-      <c r="F11" s="17"/>
-      <c r="G11" s="17"/>
-      <c r="H11" s="16"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="16"/>
+      <c r="H11" s="15"/>
       <c r="I11"/>
       <c r="J11"/>
       <c r="K11"/>
@@ -1532,18 +1564,18 @@
       <c r="AQ11"/>
     </row>
     <row r="12" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="21" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12" s="24">
+      <c r="A12" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="B12" s="22">
         <v>45950</v>
       </c>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
-      <c r="H12" s="16"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="16"/>
+      <c r="H12" s="15"/>
       <c r="I12"/>
       <c r="J12"/>
       <c r="K12"/>
@@ -1581,18 +1613,18 @@
       <c r="AQ12"/>
     </row>
     <row r="13" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="21" t="s">
-        <v>28</v>
-      </c>
-      <c r="B13" s="24">
-        <v>45988</v>
-      </c>
-      <c r="C13" s="17"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="16"/>
-      <c r="F13" s="17"/>
-      <c r="G13" s="17"/>
-      <c r="H13" s="16"/>
+      <c r="A13" s="47" t="s">
+        <v>43</v>
+      </c>
+      <c r="B13" s="49">
+        <v>45965</v>
+      </c>
+      <c r="C13" s="16"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="15"/>
+      <c r="G13" s="16"/>
+      <c r="H13" s="15"/>
       <c r="I13"/>
       <c r="J13"/>
       <c r="K13"/>
@@ -1630,14 +1662,18 @@
       <c r="AQ13"/>
     </row>
     <row r="14" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="13"/>
-      <c r="B14" s="14"/>
+      <c r="A14" s="48" t="s">
+        <v>44</v>
+      </c>
+      <c r="B14" s="49">
+        <v>45976</v>
+      </c>
       <c r="C14" s="16"/>
       <c r="D14" s="16"/>
-      <c r="E14" s="16"/>
+      <c r="E14" s="15"/>
       <c r="F14" s="16"/>
-      <c r="G14" s="16"/>
-      <c r="H14" s="16"/>
+      <c r="G14" s="15"/>
+      <c r="H14" s="15"/>
       <c r="I14"/>
       <c r="J14"/>
       <c r="K14"/>
@@ -1675,13 +1711,18 @@
       <c r="AQ14"/>
     </row>
     <row r="15" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="18"/>
+      <c r="A15" s="24" t="s">
+        <v>45</v>
+      </c>
+      <c r="B15" s="22">
+        <v>45988</v>
+      </c>
       <c r="C15" s="16"/>
       <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="16"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
       <c r="G15" s="16"/>
-      <c r="H15" s="16"/>
+      <c r="H15" s="15"/>
       <c r="I15"/>
       <c r="J15"/>
       <c r="K15"/>
@@ -1719,14 +1760,14 @@
       <c r="AQ15"/>
     </row>
     <row r="16" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="18"/>
-      <c r="B16" s="14"/>
-      <c r="C16" s="16"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="16"/>
-      <c r="G16" s="16"/>
-      <c r="H16" s="16"/>
+      <c r="A16" s="17"/>
+      <c r="B16" s="13"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="15"/>
       <c r="I16"/>
       <c r="J16"/>
       <c r="K16"/>
@@ -1764,14 +1805,14 @@
       <c r="AQ16"/>
     </row>
     <row r="17" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="18"/>
-      <c r="B17" s="14"/>
-      <c r="C17" s="16"/>
-      <c r="D17" s="16"/>
-      <c r="E17" s="16"/>
-      <c r="F17" s="16"/>
-      <c r="G17" s="16"/>
-      <c r="H17" s="16"/>
+      <c r="A17" s="17"/>
+      <c r="B17" s="13"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="15"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="15"/>
+      <c r="H17" s="15"/>
       <c r="I17"/>
       <c r="J17"/>
       <c r="K17"/>
@@ -1809,14 +1850,14 @@
       <c r="AQ17"/>
     </row>
     <row r="18" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="18"/>
-      <c r="B18" s="14"/>
-      <c r="C18" s="16"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="16"/>
-      <c r="G18" s="16"/>
-      <c r="H18" s="16"/>
+      <c r="A18" s="17"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="15"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="15"/>
+      <c r="H18" s="15"/>
       <c r="I18"/>
       <c r="J18"/>
       <c r="K18"/>
@@ -1854,16 +1895,16 @@
       <c r="AQ18"/>
     </row>
     <row r="19" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A19" s="43" t="s">
-        <v>21</v>
-      </c>
-      <c r="B19" s="43"/>
-      <c r="C19" s="43"/>
-      <c r="D19" s="43"/>
-      <c r="E19" s="43"/>
-      <c r="F19" s="43"/>
-      <c r="G19" s="43"/>
-      <c r="H19" s="43"/>
+      <c r="A19" s="33" t="s">
+        <v>20</v>
+      </c>
+      <c r="B19" s="33"/>
+      <c r="C19" s="33"/>
+      <c r="D19" s="33"/>
+      <c r="E19" s="33"/>
+      <c r="F19" s="33"/>
+      <c r="G19" s="33"/>
+      <c r="H19" s="33"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -1901,18 +1942,18 @@
       <c r="AQ19"/>
     </row>
     <row r="20" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="21" t="s">
-        <v>30</v>
-      </c>
-      <c r="B20" s="24">
+      <c r="A20" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20" s="22">
         <v>45689</v>
       </c>
-      <c r="C20" s="16"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="17"/>
-      <c r="F20" s="16"/>
-      <c r="G20" s="16"/>
-      <c r="H20" s="16"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="16"/>
+      <c r="E20" s="16"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="15"/>
+      <c r="H20" s="15"/>
       <c r="I20"/>
       <c r="J20"/>
       <c r="K20"/>
@@ -1950,18 +1991,18 @@
       <c r="AQ20"/>
     </row>
     <row r="21" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="B21" s="24">
-        <v>45689</v>
-      </c>
-      <c r="C21" s="17"/>
-      <c r="D21" s="16"/>
-      <c r="E21" s="16"/>
-      <c r="F21" s="16"/>
-      <c r="G21" s="16"/>
-      <c r="H21" s="16"/>
+      <c r="A21" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="B21" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="C21" s="16"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="15"/>
+      <c r="F21" s="15"/>
+      <c r="G21" s="15"/>
+      <c r="H21" s="15"/>
       <c r="I21"/>
       <c r="J21"/>
       <c r="K21"/>
@@ -1999,18 +2040,18 @@
       <c r="AQ21"/>
     </row>
     <row r="22" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="21" t="s">
-        <v>32</v>
-      </c>
-      <c r="B22" s="24">
-        <v>45689</v>
-      </c>
-      <c r="C22" s="16"/>
-      <c r="D22" s="16"/>
-      <c r="E22" s="16"/>
-      <c r="F22" s="16"/>
-      <c r="G22" s="17"/>
-      <c r="H22" s="16"/>
+      <c r="A22" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="B22" s="22">
+        <v>45720</v>
+      </c>
+      <c r="C22" s="15"/>
+      <c r="D22" s="15"/>
+      <c r="E22" s="15"/>
+      <c r="F22" s="15"/>
+      <c r="G22" s="16"/>
+      <c r="H22" s="15"/>
       <c r="I22"/>
       <c r="J22"/>
       <c r="K22"/>
@@ -2048,18 +2089,18 @@
       <c r="AQ22"/>
     </row>
     <row r="23" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="26" t="s">
-        <v>38</v>
-      </c>
-      <c r="B23" s="25">
-        <v>45778</v>
-      </c>
-      <c r="C23" s="17"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="16"/>
-      <c r="F23" s="17"/>
-      <c r="G23" s="17"/>
-      <c r="H23" s="16"/>
+      <c r="A23" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="B23" s="22">
+        <v>45730</v>
+      </c>
+      <c r="C23" s="16"/>
+      <c r="D23" s="16"/>
+      <c r="E23" s="15"/>
+      <c r="F23" s="16"/>
+      <c r="G23" s="16"/>
+      <c r="H23" s="15"/>
       <c r="I23"/>
       <c r="J23"/>
       <c r="K23"/>
@@ -2097,16 +2138,18 @@
       <c r="AQ23"/>
     </row>
     <row r="24" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="20" t="s">
-        <v>40</v>
-      </c>
-      <c r="B24" s="14"/>
-      <c r="C24" s="17"/>
-      <c r="D24" s="16"/>
-      <c r="E24" s="17"/>
-      <c r="F24" s="16"/>
-      <c r="G24" s="17"/>
-      <c r="H24" s="16"/>
+      <c r="A24" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="B24" s="22">
+        <v>45770</v>
+      </c>
+      <c r="C24" s="16"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="16"/>
+      <c r="F24" s="15"/>
+      <c r="G24" s="16"/>
+      <c r="H24" s="15"/>
       <c r="I24"/>
       <c r="J24"/>
       <c r="K24"/>
@@ -2144,16 +2187,18 @@
       <c r="AQ24"/>
     </row>
     <row r="25" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="49" t="s">
-        <v>42</v>
-      </c>
-      <c r="B25" s="14"/>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="16"/>
-      <c r="F25" s="16"/>
-      <c r="G25" s="17"/>
-      <c r="H25" s="16"/>
+      <c r="A25" s="26" t="s">
+        <v>37</v>
+      </c>
+      <c r="B25" s="22">
+        <v>45799</v>
+      </c>
+      <c r="C25" s="16"/>
+      <c r="D25" s="16"/>
+      <c r="E25" s="15"/>
+      <c r="F25" s="15"/>
+      <c r="G25" s="16"/>
+      <c r="H25" s="15"/>
       <c r="I25"/>
       <c r="J25"/>
       <c r="K25"/>
@@ -2191,14 +2236,14 @@
       <c r="AQ25"/>
     </row>
     <row r="26" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="23"/>
-      <c r="B26" s="14"/>
-      <c r="C26" s="16"/>
-      <c r="D26" s="16"/>
-      <c r="E26" s="16"/>
-      <c r="F26" s="16"/>
-      <c r="G26" s="16"/>
-      <c r="H26" s="16"/>
+      <c r="A26" s="21"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="15"/>
+      <c r="D26" s="15"/>
+      <c r="E26" s="15"/>
+      <c r="F26" s="15"/>
+      <c r="G26" s="15"/>
+      <c r="H26" s="15"/>
       <c r="I26"/>
       <c r="J26"/>
       <c r="K26"/>
@@ -2236,16 +2281,16 @@
       <c r="AQ26"/>
     </row>
     <row r="27" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A27" s="43" t="s">
-        <v>22</v>
-      </c>
-      <c r="B27" s="43"/>
-      <c r="C27" s="43"/>
-      <c r="D27" s="43"/>
-      <c r="E27" s="43"/>
-      <c r="F27" s="43"/>
-      <c r="G27" s="43"/>
-      <c r="H27" s="43"/>
+      <c r="A27" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="B27" s="33"/>
+      <c r="C27" s="33"/>
+      <c r="D27" s="33"/>
+      <c r="E27" s="33"/>
+      <c r="F27" s="33"/>
+      <c r="G27" s="33"/>
+      <c r="H27" s="33"/>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -2283,18 +2328,18 @@
       <c r="AQ27"/>
     </row>
     <row r="28" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="22" t="s">
-        <v>33</v>
-      </c>
-      <c r="B28" s="24">
-        <v>45536</v>
-      </c>
-      <c r="C28" s="17"/>
-      <c r="D28" s="17"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="16"/>
-      <c r="G28" s="17"/>
-      <c r="H28" s="16"/>
+      <c r="A28" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="B28" s="22">
+        <v>45914</v>
+      </c>
+      <c r="C28" s="16"/>
+      <c r="D28" s="16"/>
+      <c r="E28" s="15"/>
+      <c r="F28" s="15"/>
+      <c r="G28" s="16"/>
+      <c r="H28" s="15"/>
       <c r="I28"/>
       <c r="J28"/>
       <c r="K28"/>
@@ -2332,18 +2377,18 @@
       <c r="AQ28"/>
     </row>
     <row r="29" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="22" t="s">
-        <v>34</v>
-      </c>
-      <c r="B29" s="24">
-        <v>45536</v>
-      </c>
-      <c r="C29" s="16"/>
+      <c r="A29" s="20" t="s">
+        <v>29</v>
+      </c>
+      <c r="B29" s="22">
+        <v>45933</v>
+      </c>
+      <c r="C29" s="15"/>
       <c r="D29" s="16"/>
-      <c r="E29" s="16"/>
-      <c r="F29" s="16"/>
-      <c r="G29" s="16"/>
-      <c r="H29" s="16"/>
+      <c r="E29" s="15"/>
+      <c r="F29" s="15"/>
+      <c r="G29" s="15"/>
+      <c r="H29" s="15"/>
       <c r="I29"/>
       <c r="J29"/>
       <c r="K29"/>
@@ -2381,18 +2426,18 @@
       <c r="AQ29"/>
     </row>
     <row r="30" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="22" t="s">
-        <v>35</v>
-      </c>
-      <c r="B30" s="24">
-        <v>45536</v>
-      </c>
-      <c r="C30" s="16"/>
-      <c r="D30" s="17"/>
-      <c r="E30" s="16"/>
-      <c r="F30" s="16"/>
-      <c r="G30" s="17"/>
-      <c r="H30" s="16"/>
+      <c r="A30" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="B30" s="22">
+        <v>46348</v>
+      </c>
+      <c r="C30" s="15"/>
+      <c r="D30" s="16"/>
+      <c r="E30" s="15"/>
+      <c r="F30" s="15"/>
+      <c r="G30" s="16"/>
+      <c r="H30" s="15"/>
       <c r="I30"/>
       <c r="J30"/>
       <c r="K30"/>
@@ -2430,18 +2475,18 @@
       <c r="AQ30"/>
     </row>
     <row r="31" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="27" t="s">
-        <v>39</v>
-      </c>
-      <c r="B31" s="25">
-        <v>46001</v>
-      </c>
-      <c r="C31" s="17"/>
-      <c r="D31" s="17"/>
-      <c r="E31" s="16"/>
-      <c r="F31" s="17"/>
-      <c r="G31" s="17"/>
-      <c r="H31" s="16"/>
+      <c r="A31" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="B31" s="22">
+        <v>46363</v>
+      </c>
+      <c r="C31" s="16"/>
+      <c r="D31" s="16"/>
+      <c r="E31" s="15"/>
+      <c r="F31" s="16"/>
+      <c r="G31" s="16"/>
+      <c r="H31" s="15"/>
       <c r="I31"/>
       <c r="J31"/>
       <c r="K31"/>
@@ -2479,18 +2524,18 @@
       <c r="AQ31"/>
     </row>
     <row r="32" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="49" t="s">
-        <v>41</v>
-      </c>
-      <c r="B32" s="25">
-        <v>45947</v>
-      </c>
-      <c r="C32" s="16"/>
-      <c r="D32" s="17"/>
-      <c r="E32" s="16"/>
-      <c r="F32" s="16"/>
-      <c r="G32" s="17"/>
-      <c r="H32" s="17"/>
+      <c r="A32" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="B32" s="22">
+        <v>46374</v>
+      </c>
+      <c r="C32" s="15"/>
+      <c r="D32" s="16"/>
+      <c r="E32" s="15"/>
+      <c r="F32" s="15"/>
+      <c r="G32" s="16"/>
+      <c r="H32" s="16"/>
       <c r="I32"/>
       <c r="J32"/>
       <c r="K32"/>
@@ -2528,16 +2573,18 @@
       <c r="AQ32"/>
     </row>
     <row r="33" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="49" t="s">
-        <v>43</v>
-      </c>
-      <c r="B33" s="14"/>
-      <c r="C33" s="17"/>
-      <c r="D33" s="16"/>
-      <c r="E33" s="16"/>
-      <c r="F33" s="16"/>
-      <c r="G33" s="17"/>
-      <c r="H33" s="16"/>
+      <c r="A33" s="26" t="s">
+        <v>38</v>
+      </c>
+      <c r="B33" s="22">
+        <v>46040</v>
+      </c>
+      <c r="C33" s="16"/>
+      <c r="D33" s="15"/>
+      <c r="E33" s="15"/>
+      <c r="F33" s="15"/>
+      <c r="G33" s="16"/>
+      <c r="H33" s="15"/>
       <c r="I33"/>
       <c r="J33"/>
       <c r="K33"/>
@@ -2575,14 +2622,14 @@
       <c r="AQ33"/>
     </row>
     <row r="34" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="18"/>
-      <c r="B34" s="14"/>
-      <c r="C34" s="16"/>
-      <c r="D34" s="16"/>
-      <c r="E34" s="16"/>
-      <c r="F34" s="16"/>
-      <c r="G34" s="16"/>
-      <c r="H34" s="16"/>
+      <c r="A34" s="17"/>
+      <c r="B34" s="13"/>
+      <c r="C34" s="15"/>
+      <c r="D34" s="15"/>
+      <c r="E34" s="15"/>
+      <c r="F34" s="15"/>
+      <c r="G34" s="15"/>
+      <c r="H34" s="15"/>
       <c r="I34"/>
       <c r="J34"/>
       <c r="K34"/>
@@ -2712,6 +2759,11 @@
     <row r="81" customFormat="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
@@ -2719,11 +2771,6 @@
     <mergeCell ref="A27:H27"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>

<commit_message>
mise a jour final portefolio
</commit_message>
<xml_diff>
--- a/public/e5/annexe8-1_tableau_synthese.xlsx
+++ b/public/e5/annexe8-1_tableau_synthese.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\frani\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\frani\Portefolio\public\e5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2378B660-F7BC-4B39-9EBB-DA810F1C700D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{727145EE-3194-4DEF-8883-BA00FC037D17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="Tableau de synthèse Épreuve E5" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E5'!$A$1:$H$35</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E5'!$A$1:$H$33</definedName>
   </definedNames>
   <calcPr calcId="101716"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="50">
   <si>
     <t>Gérer le patrimoine informatique</t>
   </si>
@@ -167,26 +167,31 @@
     <t xml:space="preserve"> Elaboration de veille Technologique</t>
   </si>
   <si>
-    <t>Restructuration de l'infrastructure Stadium company (VLAN, VTP, 
-Routage inter-vlan, Routage Statique)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Infrastructure, Configuration et Administration des Services
- Informatiques de Stadium (Active Directory) </t>
-  </si>
-  <si>
-    <t>Mise en Place d'une Solution pour l'Administration à Distance Sécurisée et la Sécurisation des Interconnexions (SSH, VPN)</t>
-  </si>
-  <si>
-    <t>Solution de redondance, tolérance de panne et équilibrage de charge 
-pour les équipements réseau (HSRP, spannning-tree)</t>
-  </si>
-  <si>
-    <t>Sécurisation de l'Interconnexion du Réseau de Stadium avec Internet 
-(PfSense)</t>
-  </si>
-  <si>
-    <t>010/02/2025</t>
+    <t>2025/2026</t>
+  </si>
+  <si>
+    <t>Restructuration de l'infrastructure Stadiumcompany (VLAN, VTP, Routage inter-vlan, Routage Statique)</t>
+  </si>
+  <si>
+    <t>Sécurisation des communications entre sites et en interne (SSH/VPN/ACL/DACL/Firewall PFSENSE…)</t>
+  </si>
+  <si>
+    <t>Administration et gestion du patrimoine informatique de Stadiumcompany (OCS/GLPI)</t>
+  </si>
+  <si>
+    <t>Supervision  de l'infrastructure de Stadiumcompany (Nagios XI)</t>
+  </si>
+  <si>
+    <t>Redondance et haute disponibilité des éléments d'interconnexions de StadiumCompany (HaProxy)</t>
+  </si>
+  <si>
+    <t>Gestion et administration d'une forêt Active Directory</t>
+  </si>
+  <si>
+    <t>Mise en place portail captif pour les utilisateurs internes sous PFSENSE</t>
+  </si>
+  <si>
+    <t>Participation au suivi et aux réunions de préparation à la certification ISO 27001 de l’entreprise</t>
   </si>
 </sst>
 </file>
@@ -196,7 +201,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* &quot;-&quot;??\ [$€-1]_-"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -265,19 +270,6 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
@@ -303,7 +295,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="26">
+  <borders count="25">
     <border>
       <left/>
       <right/>
@@ -625,28 +617,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </left>
-      <right style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </right>
-      <top style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </top>
-      <bottom style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -684,9 +661,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -696,30 +670,26 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -779,15 +749,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="25" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1203,10 +1164,10 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AQ81"/>
+  <dimension ref="A1:AQ79"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="77.7109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="90.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="12.85546875" style="1" customWidth="1"/>
     <col min="3" max="8" width="18.7109375" style="1" customWidth="1"/>
     <col min="9" max="43" width="11.42578125" customWidth="1"/>
@@ -1214,56 +1175,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29" t="s">
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="29"/>
+      <c r="H1" s="26"/>
     </row>
     <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
     </row>
     <row r="3" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="39" t="s">
+      <c r="A3" s="36" t="s">
         <v>23</v>
       </c>
-      <c r="B3" s="40"/>
-      <c r="C3" s="40"/>
-      <c r="D3" s="40"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="45" t="s">
+      <c r="B3" s="37"/>
+      <c r="C3" s="37"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="38"/>
+      <c r="F3" s="42" t="s">
         <v>39</v>
       </c>
-      <c r="G3" s="40"/>
-      <c r="H3" s="46"/>
+      <c r="G3" s="37"/>
+      <c r="H3" s="43"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="42" t="s">
+      <c r="A4" s="39" t="s">
         <v>31</v>
       </c>
-      <c r="B4" s="43"/>
-      <c r="C4" s="43"/>
-      <c r="D4" s="43"/>
-      <c r="E4" s="44"/>
+      <c r="B4" s="40"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="41"/>
       <c r="F4" s="10" t="s">
         <v>8</v>
       </c>
@@ -1275,22 +1236,22 @@
       </c>
     </row>
     <row r="5" spans="1:43" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="36" t="s">
+      <c r="A5" s="33" t="s">
         <v>32</v>
       </c>
-      <c r="B5" s="37"/>
-      <c r="C5" s="37"/>
-      <c r="D5" s="37"/>
-      <c r="E5" s="37"/>
-      <c r="F5" s="37"/>
-      <c r="G5" s="37"/>
-      <c r="H5" s="38"/>
+      <c r="B5" s="34"/>
+      <c r="C5" s="34"/>
+      <c r="D5" s="34"/>
+      <c r="E5" s="34"/>
+      <c r="F5" s="34"/>
+      <c r="G5" s="34"/>
+      <c r="H5" s="35"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="27" t="s">
+      <c r="A6" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="34" t="s">
+      <c r="B6" s="31" t="s">
         <v>19</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1313,15 +1274,15 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="324.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="28"/>
-      <c r="B7" s="35"/>
+      <c r="A7" s="25"/>
+      <c r="B7" s="32"/>
       <c r="C7" s="8" t="s">
         <v>9</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="25" t="s">
+      <c r="E7" s="21" t="s">
         <v>11</v>
       </c>
       <c r="F7" s="8" t="s">
@@ -1370,16 +1331,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A8" s="30" t="s">
+      <c r="A8" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="31"/>
-      <c r="C8" s="31"/>
-      <c r="D8" s="31"/>
-      <c r="E8" s="31"/>
-      <c r="F8" s="31"/>
-      <c r="G8" s="31"/>
-      <c r="H8" s="32"/>
+      <c r="B8" s="28"/>
+      <c r="C8" s="28"/>
+      <c r="D8" s="28"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="28"/>
+      <c r="G8" s="28"/>
+      <c r="H8" s="29"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1417,18 +1378,18 @@
       <c r="AQ8"/>
     </row>
     <row r="9" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="22">
-        <v>45689</v>
-      </c>
-      <c r="C9" s="14"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="15"/>
-      <c r="F9" s="15"/>
-      <c r="G9" s="15"/>
-      <c r="H9" s="16"/>
+      <c r="B9" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C9" s="13"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14"/>
+      <c r="H9" s="15"/>
       <c r="I9"/>
       <c r="J9"/>
       <c r="K9"/>
@@ -1466,18 +1427,18 @@
       <c r="AQ9"/>
     </row>
     <row r="10" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="B10" s="22">
-        <v>45717</v>
-      </c>
-      <c r="C10" s="15"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="15"/>
-      <c r="F10" s="15"/>
-      <c r="G10" s="15"/>
-      <c r="H10" s="16"/>
+      <c r="B10" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C10" s="14"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="14"/>
+      <c r="F10" s="14"/>
+      <c r="G10" s="14"/>
+      <c r="H10" s="15"/>
       <c r="I10"/>
       <c r="J10"/>
       <c r="K10"/>
@@ -1515,18 +1476,18 @@
       <c r="AQ10"/>
     </row>
     <row r="11" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="18" t="s">
+      <c r="A11" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="B11" s="22">
-        <v>45913</v>
-      </c>
-      <c r="C11" s="16"/>
-      <c r="D11" s="15"/>
-      <c r="E11" s="15"/>
-      <c r="F11" s="16"/>
-      <c r="G11" s="16"/>
-      <c r="H11" s="15"/>
+      <c r="C11" s="14"/>
+      <c r="D11" s="14"/>
+      <c r="E11" s="14"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="14"/>
+      <c r="H11" s="14"/>
       <c r="I11"/>
       <c r="J11"/>
       <c r="K11"/>
@@ -1564,18 +1525,18 @@
       <c r="AQ11"/>
     </row>
     <row r="12" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="B12" s="22">
-        <v>45950</v>
-      </c>
-      <c r="C12" s="16"/>
-      <c r="D12" s="16"/>
-      <c r="E12" s="15"/>
-      <c r="F12" s="16"/>
-      <c r="G12" s="16"/>
-      <c r="H12" s="15"/>
+      <c r="A12" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C12" s="15"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="14"/>
+      <c r="F12" s="14"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="14"/>
       <c r="I12"/>
       <c r="J12"/>
       <c r="K12"/>
@@ -1613,18 +1574,18 @@
       <c r="AQ12"/>
     </row>
     <row r="13" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="47" t="s">
-        <v>43</v>
-      </c>
-      <c r="B13" s="49">
-        <v>45965</v>
-      </c>
-      <c r="C13" s="16"/>
+      <c r="A13" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="B13" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C13" s="15"/>
       <c r="D13" s="15"/>
-      <c r="E13" s="15"/>
-      <c r="F13" s="15"/>
-      <c r="G13" s="16"/>
-      <c r="H13" s="15"/>
+      <c r="E13" s="14"/>
+      <c r="F13" s="14"/>
+      <c r="G13" s="15"/>
+      <c r="H13" s="14"/>
       <c r="I13"/>
       <c r="J13"/>
       <c r="K13"/>
@@ -1662,18 +1623,18 @@
       <c r="AQ13"/>
     </row>
     <row r="14" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="48" t="s">
-        <v>44</v>
-      </c>
-      <c r="B14" s="49">
-        <v>45976</v>
-      </c>
-      <c r="C14" s="16"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="15"/>
-      <c r="F14" s="16"/>
-      <c r="G14" s="15"/>
-      <c r="H14" s="15"/>
+      <c r="A14" s="23" t="s">
+        <v>45</v>
+      </c>
+      <c r="B14" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C14" s="14"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="14"/>
+      <c r="F14" s="14"/>
+      <c r="G14" s="14"/>
+      <c r="H14" s="14"/>
       <c r="I14"/>
       <c r="J14"/>
       <c r="K14"/>
@@ -1711,18 +1672,18 @@
       <c r="AQ14"/>
     </row>
     <row r="15" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="24" t="s">
-        <v>45</v>
-      </c>
-      <c r="B15" s="22">
-        <v>45988</v>
-      </c>
-      <c r="C15" s="16"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="15"/>
+      <c r="A15" s="20" t="s">
+        <v>46</v>
+      </c>
+      <c r="B15" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C15" s="15"/>
+      <c r="D15" s="14"/>
+      <c r="E15" s="14"/>
       <c r="F15" s="15"/>
-      <c r="G15" s="16"/>
-      <c r="H15" s="15"/>
+      <c r="G15" s="14"/>
+      <c r="H15" s="14"/>
       <c r="I15"/>
       <c r="J15"/>
       <c r="K15"/>
@@ -1760,14 +1721,18 @@
       <c r="AQ15"/>
     </row>
     <row r="16" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="17"/>
-      <c r="B16" s="13"/>
-      <c r="C16" s="15"/>
+      <c r="A16" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="B16" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C16" s="14"/>
       <c r="D16" s="15"/>
-      <c r="E16" s="15"/>
+      <c r="E16" s="14"/>
       <c r="F16" s="15"/>
       <c r="G16" s="15"/>
-      <c r="H16" s="15"/>
+      <c r="H16" s="14"/>
       <c r="I16"/>
       <c r="J16"/>
       <c r="K16"/>
@@ -1805,14 +1770,18 @@
       <c r="AQ16"/>
     </row>
     <row r="17" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="17"/>
-      <c r="B17" s="13"/>
-      <c r="C17" s="15"/>
-      <c r="D17" s="15"/>
-      <c r="E17" s="15"/>
-      <c r="F17" s="15"/>
+      <c r="A17" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="B17" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C17" s="14"/>
+      <c r="D17" s="14"/>
+      <c r="E17" s="14"/>
+      <c r="F17" s="14"/>
       <c r="G17" s="15"/>
-      <c r="H17" s="15"/>
+      <c r="H17" s="14"/>
       <c r="I17"/>
       <c r="J17"/>
       <c r="K17"/>
@@ -1849,15 +1818,17 @@
       <c r="AP17"/>
       <c r="AQ17"/>
     </row>
-    <row r="18" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="17"/>
-      <c r="B18" s="13"/>
-      <c r="C18" s="15"/>
-      <c r="D18" s="15"/>
-      <c r="E18" s="15"/>
-      <c r="F18" s="15"/>
-      <c r="G18" s="15"/>
-      <c r="H18" s="15"/>
+    <row r="18" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
+      <c r="A18" s="30" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" s="30"/>
+      <c r="C18" s="30"/>
+      <c r="D18" s="30"/>
+      <c r="E18" s="30"/>
+      <c r="F18" s="30"/>
+      <c r="G18" s="30"/>
+      <c r="H18" s="30"/>
       <c r="I18"/>
       <c r="J18"/>
       <c r="K18"/>
@@ -1894,17 +1865,19 @@
       <c r="AP18"/>
       <c r="AQ18"/>
     </row>
-    <row r="19" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A19" s="33" t="s">
-        <v>20</v>
-      </c>
-      <c r="B19" s="33"/>
-      <c r="C19" s="33"/>
-      <c r="D19" s="33"/>
-      <c r="E19" s="33"/>
-      <c r="F19" s="33"/>
-      <c r="G19" s="33"/>
-      <c r="H19" s="33"/>
+    <row r="19" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B19" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C19" s="14"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="14"/>
+      <c r="G19" s="14"/>
+      <c r="H19" s="14"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -1942,18 +1915,18 @@
       <c r="AQ19"/>
     </row>
     <row r="20" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="B20" s="22">
-        <v>45689</v>
+      <c r="A20" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="18" t="s">
+        <v>41</v>
       </c>
       <c r="C20" s="15"/>
-      <c r="D20" s="16"/>
-      <c r="E20" s="16"/>
-      <c r="F20" s="15"/>
-      <c r="G20" s="15"/>
-      <c r="H20" s="15"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="14"/>
+      <c r="G20" s="14"/>
+      <c r="H20" s="14"/>
       <c r="I20"/>
       <c r="J20"/>
       <c r="K20"/>
@@ -1991,18 +1964,18 @@
       <c r="AQ20"/>
     </row>
     <row r="21" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="B21" s="22" t="s">
-        <v>46</v>
-      </c>
-      <c r="C21" s="16"/>
-      <c r="D21" s="15"/>
-      <c r="E21" s="15"/>
-      <c r="F21" s="15"/>
+      <c r="A21" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B21" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C21" s="14"/>
+      <c r="D21" s="14"/>
+      <c r="E21" s="14"/>
+      <c r="F21" s="14"/>
       <c r="G21" s="15"/>
-      <c r="H21" s="15"/>
+      <c r="H21" s="14"/>
       <c r="I21"/>
       <c r="J21"/>
       <c r="K21"/>
@@ -2041,17 +2014,17 @@
     </row>
     <row r="22" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="19" t="s">
-        <v>27</v>
-      </c>
-      <c r="B22" s="22">
-        <v>45720</v>
+        <v>33</v>
+      </c>
+      <c r="B22" s="18" t="s">
+        <v>41</v>
       </c>
       <c r="C22" s="15"/>
       <c r="D22" s="15"/>
-      <c r="E22" s="15"/>
+      <c r="E22" s="14"/>
       <c r="F22" s="15"/>
-      <c r="G22" s="16"/>
-      <c r="H22" s="15"/>
+      <c r="G22" s="15"/>
+      <c r="H22" s="14"/>
       <c r="I22"/>
       <c r="J22"/>
       <c r="K22"/>
@@ -2089,18 +2062,18 @@
       <c r="AQ22"/>
     </row>
     <row r="23" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="B23" s="22">
-        <v>45730</v>
-      </c>
-      <c r="C23" s="16"/>
-      <c r="D23" s="16"/>
+      <c r="A23" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="B23" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C23" s="15"/>
+      <c r="D23" s="14"/>
       <c r="E23" s="15"/>
-      <c r="F23" s="16"/>
-      <c r="G23" s="16"/>
-      <c r="H23" s="15"/>
+      <c r="F23" s="14"/>
+      <c r="G23" s="15"/>
+      <c r="H23" s="14"/>
       <c r="I23"/>
       <c r="J23"/>
       <c r="K23"/>
@@ -2138,18 +2111,18 @@
       <c r="AQ23"/>
     </row>
     <row r="24" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="B24" s="22">
-        <v>45770</v>
-      </c>
-      <c r="C24" s="16"/>
+      <c r="A24" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="B24" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C24" s="15"/>
       <c r="D24" s="15"/>
-      <c r="E24" s="16"/>
-      <c r="F24" s="15"/>
-      <c r="G24" s="16"/>
-      <c r="H24" s="15"/>
+      <c r="E24" s="14"/>
+      <c r="F24" s="14"/>
+      <c r="G24" s="15"/>
+      <c r="H24" s="14"/>
       <c r="I24"/>
       <c r="J24"/>
       <c r="K24"/>
@@ -2186,19 +2159,17 @@
       <c r="AP24"/>
       <c r="AQ24"/>
     </row>
-    <row r="25" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="26" t="s">
-        <v>37</v>
-      </c>
-      <c r="B25" s="22">
-        <v>45799</v>
-      </c>
-      <c r="C25" s="16"/>
-      <c r="D25" s="16"/>
-      <c r="E25" s="15"/>
-      <c r="F25" s="15"/>
-      <c r="G25" s="16"/>
-      <c r="H25" s="15"/>
+    <row r="25" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
+      <c r="A25" s="30" t="s">
+        <v>21</v>
+      </c>
+      <c r="B25" s="30"/>
+      <c r="C25" s="30"/>
+      <c r="D25" s="30"/>
+      <c r="E25" s="30"/>
+      <c r="F25" s="30"/>
+      <c r="G25" s="30"/>
+      <c r="H25" s="30"/>
       <c r="I25"/>
       <c r="J25"/>
       <c r="K25"/>
@@ -2236,14 +2207,18 @@
       <c r="AQ25"/>
     </row>
     <row r="26" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="21"/>
-      <c r="B26" s="13"/>
+      <c r="A26" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" s="18" t="s">
+        <v>41</v>
+      </c>
       <c r="C26" s="15"/>
       <c r="D26" s="15"/>
-      <c r="E26" s="15"/>
-      <c r="F26" s="15"/>
+      <c r="E26" s="14"/>
+      <c r="F26" s="14"/>
       <c r="G26" s="15"/>
-      <c r="H26" s="15"/>
+      <c r="H26" s="14"/>
       <c r="I26"/>
       <c r="J26"/>
       <c r="K26"/>
@@ -2280,17 +2255,19 @@
       <c r="AP26"/>
       <c r="AQ26"/>
     </row>
-    <row r="27" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A27" s="33" t="s">
-        <v>21</v>
-      </c>
-      <c r="B27" s="33"/>
-      <c r="C27" s="33"/>
-      <c r="D27" s="33"/>
-      <c r="E27" s="33"/>
-      <c r="F27" s="33"/>
-      <c r="G27" s="33"/>
-      <c r="H27" s="33"/>
+    <row r="27" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C27" s="14"/>
+      <c r="D27" s="15"/>
+      <c r="E27" s="14"/>
+      <c r="F27" s="14"/>
+      <c r="G27" s="14"/>
+      <c r="H27" s="14"/>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -2328,18 +2305,18 @@
       <c r="AQ27"/>
     </row>
     <row r="28" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="20" t="s">
-        <v>28</v>
-      </c>
-      <c r="B28" s="22">
-        <v>45914</v>
-      </c>
-      <c r="C28" s="16"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="15"/>
-      <c r="F28" s="15"/>
-      <c r="G28" s="16"/>
-      <c r="H28" s="15"/>
+      <c r="A28" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C28" s="14"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="14"/>
+      <c r="F28" s="14"/>
+      <c r="G28" s="15"/>
+      <c r="H28" s="14"/>
       <c r="I28"/>
       <c r="J28"/>
       <c r="K28"/>
@@ -2378,17 +2355,17 @@
     </row>
     <row r="29" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="B29" s="22">
-        <v>45933</v>
+        <v>34</v>
+      </c>
+      <c r="B29" s="18" t="s">
+        <v>41</v>
       </c>
       <c r="C29" s="15"/>
-      <c r="D29" s="16"/>
-      <c r="E29" s="15"/>
+      <c r="D29" s="15"/>
+      <c r="E29" s="14"/>
       <c r="F29" s="15"/>
       <c r="G29" s="15"/>
-      <c r="H29" s="15"/>
+      <c r="H29" s="14"/>
       <c r="I29"/>
       <c r="J29"/>
       <c r="K29"/>
@@ -2426,17 +2403,17 @@
       <c r="AQ29"/>
     </row>
     <row r="30" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="B30" s="22">
-        <v>46348</v>
-      </c>
-      <c r="C30" s="15"/>
-      <c r="D30" s="16"/>
-      <c r="E30" s="15"/>
-      <c r="F30" s="15"/>
-      <c r="G30" s="16"/>
+      <c r="A30" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="B30" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C30" s="14"/>
+      <c r="D30" s="15"/>
+      <c r="E30" s="14"/>
+      <c r="F30" s="14"/>
+      <c r="G30" s="15"/>
       <c r="H30" s="15"/>
       <c r="I30"/>
       <c r="J30"/>
@@ -2475,18 +2452,18 @@
       <c r="AQ30"/>
     </row>
     <row r="31" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="24" t="s">
-        <v>34</v>
-      </c>
-      <c r="B31" s="22">
-        <v>46363</v>
-      </c>
-      <c r="C31" s="16"/>
-      <c r="D31" s="16"/>
-      <c r="E31" s="15"/>
-      <c r="F31" s="16"/>
-      <c r="G31" s="16"/>
-      <c r="H31" s="15"/>
+      <c r="A31" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="B31" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C31" s="15"/>
+      <c r="D31" s="14"/>
+      <c r="E31" s="14"/>
+      <c r="F31" s="14"/>
+      <c r="G31" s="15"/>
+      <c r="H31" s="14"/>
       <c r="I31"/>
       <c r="J31"/>
       <c r="K31"/>
@@ -2524,18 +2501,18 @@
       <c r="AQ31"/>
     </row>
     <row r="32" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="B32" s="22">
-        <v>46374</v>
-      </c>
-      <c r="C32" s="15"/>
-      <c r="D32" s="16"/>
-      <c r="E32" s="15"/>
+      <c r="A32" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="B32" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C32" s="14"/>
+      <c r="D32" s="14"/>
+      <c r="E32" s="14"/>
       <c r="F32" s="15"/>
-      <c r="G32" s="16"/>
-      <c r="H32" s="16"/>
+      <c r="G32" s="14"/>
+      <c r="H32" s="15"/>
       <c r="I32"/>
       <c r="J32"/>
       <c r="K32"/>
@@ -2572,19 +2549,15 @@
       <c r="AP32"/>
       <c r="AQ32"/>
     </row>
-    <row r="33" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="26" t="s">
-        <v>38</v>
-      </c>
-      <c r="B33" s="22">
-        <v>46040</v>
-      </c>
-      <c r="C33" s="16"/>
-      <c r="D33" s="15"/>
-      <c r="E33" s="15"/>
-      <c r="F33" s="15"/>
-      <c r="G33" s="16"/>
-      <c r="H33" s="15"/>
+    <row r="33" spans="1:43" s="2" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A33" s="5"/>
+      <c r="B33" s="3"/>
+      <c r="C33" s="4"/>
+      <c r="D33" s="4"/>
+      <c r="E33" s="4"/>
+      <c r="F33" s="4"/>
+      <c r="G33" s="4"/>
+      <c r="H33" s="4"/>
       <c r="I33"/>
       <c r="J33"/>
       <c r="K33"/>
@@ -2621,96 +2594,8 @@
       <c r="AP33"/>
       <c r="AQ33"/>
     </row>
-    <row r="34" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="17"/>
-      <c r="B34" s="13"/>
-      <c r="C34" s="15"/>
-      <c r="D34" s="15"/>
-      <c r="E34" s="15"/>
-      <c r="F34" s="15"/>
-      <c r="G34" s="15"/>
-      <c r="H34" s="15"/>
-      <c r="I34"/>
-      <c r="J34"/>
-      <c r="K34"/>
-      <c r="L34"/>
-      <c r="M34"/>
-      <c r="N34"/>
-      <c r="O34"/>
-      <c r="P34"/>
-      <c r="Q34"/>
-      <c r="R34"/>
-      <c r="S34"/>
-      <c r="T34"/>
-      <c r="U34"/>
-      <c r="V34"/>
-      <c r="W34"/>
-      <c r="X34"/>
-      <c r="Y34"/>
-      <c r="Z34"/>
-      <c r="AA34"/>
-      <c r="AB34"/>
-      <c r="AC34"/>
-      <c r="AD34"/>
-      <c r="AE34"/>
-      <c r="AF34"/>
-      <c r="AG34"/>
-      <c r="AH34"/>
-      <c r="AI34"/>
-      <c r="AJ34"/>
-      <c r="AK34"/>
-      <c r="AL34"/>
-      <c r="AM34"/>
-      <c r="AN34"/>
-      <c r="AO34"/>
-      <c r="AP34"/>
-      <c r="AQ34"/>
-    </row>
-    <row r="35" spans="1:43" s="2" customFormat="1" ht="15" x14ac:dyDescent="0.2">
-      <c r="A35" s="5"/>
-      <c r="B35" s="3"/>
-      <c r="C35" s="4"/>
-      <c r="D35" s="4"/>
-      <c r="E35" s="4"/>
-      <c r="F35" s="4"/>
-      <c r="G35" s="4"/>
-      <c r="H35" s="4"/>
-      <c r="I35"/>
-      <c r="J35"/>
-      <c r="K35"/>
-      <c r="L35"/>
-      <c r="M35"/>
-      <c r="N35"/>
-      <c r="O35"/>
-      <c r="P35"/>
-      <c r="Q35"/>
-      <c r="R35"/>
-      <c r="S35"/>
-      <c r="T35"/>
-      <c r="U35"/>
-      <c r="V35"/>
-      <c r="W35"/>
-      <c r="X35"/>
-      <c r="Y35"/>
-      <c r="Z35"/>
-      <c r="AA35"/>
-      <c r="AB35"/>
-      <c r="AC35"/>
-      <c r="AD35"/>
-      <c r="AE35"/>
-      <c r="AF35"/>
-      <c r="AG35"/>
-      <c r="AH35"/>
-      <c r="AI35"/>
-      <c r="AJ35"/>
-      <c r="AK35"/>
-      <c r="AL35"/>
-      <c r="AM35"/>
-      <c r="AN35"/>
-      <c r="AO35"/>
-      <c r="AP35"/>
-      <c r="AQ35"/>
-    </row>
+    <row r="34" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="35" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="36" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="37" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="38" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
@@ -2755,8 +2640,6 @@
     <row r="77" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="78" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="79" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="80" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="81" customFormat="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="12">
     <mergeCell ref="G1:H1"/>
@@ -2767,8 +2650,8 @@
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A19:H19"/>
-    <mergeCell ref="A27:H27"/>
+    <mergeCell ref="A18:H18"/>
+    <mergeCell ref="A25:H25"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
   </mergeCells>

</xml_diff>